<commit_message>
feat: add remaining project files (api client, routing, inventory, dist build)
Include all unstaged changes that were missing from previous commits:
- src/api/client.ts — inventory + schedule AI endpoints
- src/index.tsx, Navigation.tsx, Frame.tsx — routing for new pages
- src/screens/SalonCRM/index.ts — export InventoryPage, SpectraPreviewPage
- src/screens/StockGrid/ — new StockGrid page
- netlify/functions/inventory.js — inventory API function (Neon)
- migrations/15_inventory.sql — inventory table schema
- dist/ — updated production build assets
- Footer.tsx, stats.html — minor updates
</commit_message>
<xml_diff>
--- a/reports/jan-2025-vs-jan-2026-salons.xlsx
+++ b/reports/jan-2025-vs-jan-2026-salons.xlsx
@@ -1,41 +1,230 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maorganon/Downloads/spectra-salon-website-main/reports/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74EF97AA-0619-7840-A9A5-1680A5A488DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="760" windowWidth="18520" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Jan25_vs_Jan26" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Jan25_vs_Jan26!$A$1:$E$1</definedName>
+  </definedNames>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+  <si>
+    <t>DisplayName</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Jan 2025</t>
+  </si>
+  <si>
+    <t>Jan 2026</t>
+  </si>
+  <si>
+    <t>% Change</t>
+  </si>
+  <si>
+    <t>לא נמצא</t>
+  </si>
+  <si>
+    <t>#9232</t>
+  </si>
+  <si>
+    <t>יואל ברמי</t>
+  </si>
+  <si>
+    <t>#5715</t>
+  </si>
+  <si>
+    <t>רוזאן חבקה</t>
+  </si>
+  <si>
+    <t>#9149</t>
+  </si>
+  <si>
+    <t>שראל לגזיאל</t>
+  </si>
+  <si>
+    <t>#8750</t>
+  </si>
+  <si>
+    <t>האחים סונגו</t>
+  </si>
+  <si>
+    <t>#1194</t>
+  </si>
+  <si>
+    <t>אלי יוסף</t>
+  </si>
+  <si>
+    <t>#5583</t>
+  </si>
+  <si>
+    <t>דודו ורועי</t>
+  </si>
+  <si>
+    <t>#0554</t>
+  </si>
+  <si>
+    <t>הקומה 10</t>
+  </si>
+  <si>
+    <t>#6235</t>
+  </si>
+  <si>
+    <t>עידן</t>
+  </si>
+  <si>
+    <t>#9913</t>
+  </si>
+  <si>
+    <t>דקל סבן</t>
+  </si>
+  <si>
+    <t>#7280</t>
+  </si>
+  <si>
+    <t>אריאל אסולין</t>
+  </si>
+  <si>
+    <t>#7031</t>
+  </si>
+  <si>
+    <t>ירון נחמיאס</t>
+  </si>
+  <si>
+    <t>#0501</t>
+  </si>
+  <si>
+    <t>Maor Ganon</t>
+  </si>
+  <si>
+    <t>#8613</t>
+  </si>
+  <si>
+    <t>איציק קירמה</t>
+  </si>
+  <si>
+    <t>#2362</t>
+  </si>
+  <si>
+    <t>אלמוג כהן</t>
+  </si>
+  <si>
+    <t>#5719</t>
+  </si>
+  <si>
+    <t>רועי לוי עיצוב שיער</t>
+  </si>
+  <si>
+    <t>#5330</t>
+  </si>
+  <si>
+    <t>יקיר כהן - ספר על הבר</t>
+  </si>
+  <si>
+    <t>#7122</t>
+  </si>
+  <si>
+    <t>סלון שמלי</t>
+  </si>
+  <si>
+    <t>#8252</t>
+  </si>
+  <si>
+    <t>מעיין ששון</t>
+  </si>
+  <si>
+    <t>#2837</t>
+  </si>
+  <si>
+    <t>אלברט אלימוב</t>
+  </si>
+  <si>
+    <t>#4836</t>
+  </si>
+  <si>
+    <t>Vol. סלון</t>
+  </si>
+  <si>
+    <t>#5149</t>
+  </si>
+  <si>
+    <t>מאווה מור יוסף</t>
+  </si>
+  <si>
+    <t>#7995</t>
+  </si>
+  <si>
+    <t>אירה</t>
+  </si>
+  <si>
+    <t>#0820</t>
+  </si>
+  <si>
+    <t>ג׳וני בראון</t>
+  </si>
+  <si>
+    <t>#9684</t>
+  </si>
+  <si>
+    <t>אבי פולדי</t>
+  </si>
+  <si>
+    <t>#9896</t>
+  </si>
+  <si>
+    <t>לילה רויפמן</t>
+  </si>
+  <si>
+    <t>#8608</t>
+  </si>
+  <si>
+    <t>הדר חדד</t>
+  </si>
+  <si>
+    <t>#3696</t>
+  </si>
+  <si>
+    <t>אהדס - נס ציונה</t>
+  </si>
+  <si>
+    <t>#1221</t>
+  </si>
+  <si>
+    <t>בן יפרח</t>
+  </si>
+  <si>
+    <t>#4896</t>
+  </si>
+  <si>
+    <t>שחר אפוטה</t>
+  </si>
+  <si>
+    <t>#7276</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -43,13 +232,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -64,14 +265,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,32 +606,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="15" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>DisplayName</v>
-      </c>
-      <c r="B1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Jan 2025</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Jan 2026</v>
-      </c>
-      <c r="E1" t="str">
-        <v>% Change</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>לא נמצא</v>
-      </c>
-      <c r="B2" t="str">
-        <v>#9232</v>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
       </c>
       <c r="C2">
         <v>2179</v>
@@ -433,12 +644,12 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>יואל ברמי</v>
-      </c>
-      <c r="B3" t="str">
-        <v>#5715</v>
+    <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
       <c r="C3">
         <v>2592</v>
@@ -450,12 +661,12 @@
         <v>-92.9</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>רוזאן חבקה</v>
-      </c>
-      <c r="B4" t="str">
-        <v>#9149</v>
+    <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
       </c>
       <c r="C4">
         <v>985</v>
@@ -467,12 +678,12 @@
         <v>-92.6</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>שראל לגזיאל</v>
-      </c>
-      <c r="B5" t="str">
-        <v>#8750</v>
+    <row r="5" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
       </c>
       <c r="C5">
         <v>17458</v>
@@ -484,12 +695,12 @@
         <v>-79.2</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>האחים סונגו</v>
-      </c>
-      <c r="B6" t="str">
-        <v>#1194</v>
+    <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
       </c>
       <c r="C6">
         <v>24518</v>
@@ -501,12 +712,12 @@
         <v>-77.7</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>אלי יוסף</v>
-      </c>
-      <c r="B7" t="str">
-        <v>#5583</v>
+    <row r="7" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
       </c>
       <c r="C7">
         <v>6167</v>
@@ -518,12 +729,12 @@
         <v>-51.4</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>דודו ורועי</v>
-      </c>
-      <c r="B8" t="str">
-        <v>#0554</v>
+    <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
       </c>
       <c r="C8">
         <v>1391</v>
@@ -535,12 +746,12 @@
         <v>-50.7</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>הקומה 10</v>
-      </c>
-      <c r="B9" t="str">
-        <v>#6235</v>
+    <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
       </c>
       <c r="C9">
         <v>31431</v>
@@ -552,12 +763,12 @@
         <v>-45.6</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>עידן</v>
-      </c>
-      <c r="B10" t="str">
-        <v>#9913</v>
+    <row r="10" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
       </c>
       <c r="C10">
         <v>1531</v>
@@ -569,12 +780,12 @@
         <v>-45.2</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>דקל סבן</v>
-      </c>
-      <c r="B11" t="str">
-        <v>#7280</v>
+    <row r="11" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
       </c>
       <c r="C11">
         <v>1359</v>
@@ -586,12 +797,12 @@
         <v>-45.2</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>אריאל אסולין</v>
-      </c>
-      <c r="B12" t="str">
-        <v>#7031</v>
+    <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
       </c>
       <c r="C12">
         <v>18646</v>
@@ -603,12 +814,12 @@
         <v>-44.7</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>ירון נחמיאס</v>
-      </c>
-      <c r="B13" t="str">
-        <v>#0501</v>
+    <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
       </c>
       <c r="C13">
         <v>11005</v>
@@ -620,12 +831,12 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Maor Ganon</v>
-      </c>
-      <c r="B14" t="str">
-        <v>#8613</v>
+    <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
       </c>
       <c r="C14">
         <v>5213</v>
@@ -634,15 +845,15 @@
         <v>3145</v>
       </c>
       <c r="E14">
-        <v>-39.7</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>איציק קירמה</v>
-      </c>
-      <c r="B15" t="str">
-        <v>#2362</v>
+        <v>-39.700000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
       </c>
       <c r="C15">
         <v>17196</v>
@@ -654,12 +865,12 @@
         <v>-36.5</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>אלמוג כהן</v>
-      </c>
-      <c r="B16" t="str">
-        <v>#5719</v>
+    <row r="16" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
       </c>
       <c r="C16">
         <v>3445</v>
@@ -671,12 +882,12 @@
         <v>-35.5</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>רועי לוי עיצוב שיער</v>
-      </c>
-      <c r="B17" t="str">
-        <v>#5330</v>
+    <row r="17" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
+        <v>36</v>
       </c>
       <c r="C17">
         <v>1630</v>
@@ -685,15 +896,15 @@
         <v>1056</v>
       </c>
       <c r="E17">
-        <v>-35.2</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>יקיר כהן - ספר על הבר</v>
-      </c>
-      <c r="B18" t="str">
-        <v>#7122</v>
+        <v>-35.200000000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
       </c>
       <c r="C18">
         <v>6078</v>
@@ -705,12 +916,12 @@
         <v>-33.1</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>סלון שמלי</v>
-      </c>
-      <c r="B19" t="str">
-        <v>#8252</v>
+    <row r="19" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
       </c>
       <c r="C19">
         <v>21061</v>
@@ -722,12 +933,12 @@
         <v>-33.1</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>מעיין ששון</v>
-      </c>
-      <c r="B20" t="str">
-        <v>#2837</v>
+    <row r="20" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
       </c>
       <c r="C20">
         <v>3299</v>
@@ -739,12 +950,12 @@
         <v>-30</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>אלברט אלימוב</v>
-      </c>
-      <c r="B21" t="str">
-        <v>#4836</v>
+    <row r="21" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
       </c>
       <c r="C21">
         <v>2017</v>
@@ -753,15 +964,15 @@
         <v>1636</v>
       </c>
       <c r="E21">
-        <v>-18.9</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Vol. סלון</v>
-      </c>
-      <c r="B22" t="str">
-        <v>#5149</v>
+        <v>-18.899999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" t="s">
+        <v>46</v>
       </c>
       <c r="C22">
         <v>6178</v>
@@ -770,15 +981,15 @@
         <v>5100</v>
       </c>
       <c r="E22">
-        <v>-17.4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>מאווה מור יוסף</v>
-      </c>
-      <c r="B23" t="str">
-        <v>#7995</v>
+        <v>-17.399999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="s">
+        <v>48</v>
       </c>
       <c r="C23">
         <v>13446</v>
@@ -790,12 +1001,12 @@
         <v>-17.3</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>אירה</v>
-      </c>
-      <c r="B24" t="str">
-        <v>#0820</v>
+    <row r="24" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" t="s">
+        <v>50</v>
       </c>
       <c r="C24">
         <v>4183</v>
@@ -807,12 +1018,12 @@
         <v>-17</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>ג׳וני בראון</v>
-      </c>
-      <c r="B25" t="str">
-        <v>#9684</v>
+    <row r="25" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" t="s">
+        <v>52</v>
       </c>
       <c r="C25">
         <v>4869</v>
@@ -824,12 +1035,12 @@
         <v>-16.7</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>אבי פולדי</v>
-      </c>
-      <c r="B26" t="str">
-        <v>#9896</v>
+    <row r="26" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" t="s">
+        <v>54</v>
       </c>
       <c r="C26">
         <v>9500</v>
@@ -841,12 +1052,12 @@
         <v>-15.9</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>לילה רויפמן</v>
-      </c>
-      <c r="B27" t="str">
-        <v>#8608</v>
+    <row r="27" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
       </c>
       <c r="C27">
         <v>2502</v>
@@ -858,12 +1069,12 @@
         <v>-15.5</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>הדר חדד</v>
-      </c>
-      <c r="B28" t="str">
-        <v>#3696</v>
+    <row r="28" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" t="s">
+        <v>58</v>
       </c>
       <c r="C28">
         <v>3895</v>
@@ -875,12 +1086,12 @@
         <v>-13.3</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>אהדס - נס ציונה</v>
-      </c>
-      <c r="B29" t="str">
-        <v>#1221</v>
+    <row r="29" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" t="s">
+        <v>60</v>
       </c>
       <c r="C29">
         <v>9641</v>
@@ -892,12 +1103,12 @@
         <v>-12.9</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>בן יפרח</v>
-      </c>
-      <c r="B30" t="str">
-        <v>#4896</v>
+    <row r="30" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" t="s">
+        <v>62</v>
       </c>
       <c r="C30">
         <v>20615</v>
@@ -909,12 +1120,12 @@
         <v>-12.9</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>שחר אפוטה</v>
-      </c>
-      <c r="B31" t="str">
-        <v>#7276</v>
+    <row r="31" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" t="s">
+        <v>64</v>
       </c>
       <c r="C31">
         <v>4875</v>
@@ -927,8 +1138,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
+    <ignoredError sqref="A1:E31" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>